<commit_message>
scan: seg7 2026-07-10 18:27 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq8_2026-07-09.xlsx
+++ b/output/full_scan/batch_seq8_2026-07-09.xlsx
@@ -1754,21 +1754,21 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>6928</v>
+        <v>7402</v>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>攸泰科技</t>
+          <t>邑錡</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
         <v/>
       </c>
       <c r="D25" s="2" t="n">
-        <v>660.356434821952</v>
+        <v>657.9599836910082</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>53.3</v>
+        <v>131</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
@@ -1779,13 +1779,13 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>57.63566193007057</v>
+        <v>63.74607051890244</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>32.03870086834914</v>
+        <v>31.87193742892348</v>
       </c>
       <c r="J25" s="2" t="n">
-        <v>0.4347882539286762</v>
+        <v>1.895998369100822</v>
       </c>
       <c r="K25" s="2" t="n">
         <v>0</v>
@@ -1797,31 +1797,31 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>0.3178441433848018</v>
+        <v>3.251686895042466</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>volume_break, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>7402</v>
+        <v>6965</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>邑錡</t>
+          <t>中傑-KY</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
         <v/>
       </c>
       <c r="D26" s="2" t="n">
-        <v>657.9599836910082</v>
+        <v>657.1843931304295</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>131</v>
+        <v>80</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
@@ -1832,16 +1832,16 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>63.74607051890244</v>
+        <v>52.20498622387128</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>31.87193742892348</v>
+        <v>22.25081504807666</v>
       </c>
       <c r="J26" s="2" t="n">
-        <v>1.895998369100822</v>
+        <v>0.5680626029119896</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L26" s="2" t="n">
         <v>0</v>
@@ -1850,31 +1850,31 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>3.251686895042466</v>
+        <v>0.151930499100081</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>volume_break, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, mfi_strong, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>6965</v>
+        <v>6890</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>中傑-KY</t>
+          <t>來億-KY</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
         <v/>
       </c>
       <c r="D27" s="2" t="n">
-        <v>657.1843931304295</v>
+        <v>655.1476617649607</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>80</v>
+        <v>206</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
@@ -1885,49 +1885,49 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>52.20498622387128</v>
+        <v>47.04697220223746</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>22.25081504807666</v>
+        <v>18.8247603452546</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>0.5680626029119896</v>
+        <v>0.9427276747293294</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M27" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>0.151930499100081</v>
+        <v>-4.348860042339972</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, liquidity_ok, stronger_than_market, kd_golden_cross, obv_uptrend, invest_trust_buy_2d, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>6890</v>
+        <v>7717</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>來億-KY</t>
+          <t>萊德光電-KY</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v/>
       </c>
       <c r="D28" s="2" t="n">
-        <v>655.1476617649607</v>
+        <v>652.2429131338725</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>206</v>
+        <v>422.5</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -1938,49 +1938,49 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>47.04697220223746</v>
+        <v>32.03154027332101</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>18.8247603452546</v>
+        <v>22.98215457332702</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>0.9427276747293294</v>
+        <v>0.2816613219084758</v>
       </c>
       <c r="K28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L28" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M28" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>-4.348860042339972</v>
+        <v>0.6582596039140114</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, liquidity_ok, stronger_than_market, kd_golden_cross, obv_uptrend, invest_trust_buy_2d, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, hist_turn_positive, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>7717</v>
+        <v>6928</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>萊德光電-KY</t>
+          <t>攸泰科技</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
         <v/>
       </c>
       <c r="D29" s="2" t="n">
-        <v>652.2429131338725</v>
+        <v>640.356434821952</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>422.5</v>
+        <v>53.3</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
@@ -1991,13 +1991,13 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>32.03154027332101</v>
+        <v>57.63566193007057</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>22.98215457332702</v>
+        <v>32.03870086834914</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>0.2816613219084758</v>
+        <v>0.4347882539286762</v>
       </c>
       <c r="K29" s="2" t="n">
         <v>0</v>
@@ -2009,11 +2009,11 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>0.6582596039140114</v>
+        <v>0.3178441433848018</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, hist_turn_positive, adx_trending, stronger_than_market</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -2125,21 +2125,21 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>7799</v>
+        <v>6869</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>禾榮科</t>
+          <t>雲豹能源</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>611.7499454937273</v>
+        <v>626.663640477753</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>435.5</v>
+        <v>71.2</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -2150,16 +2150,16 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>60.12411481233664</v>
+        <v>38.86067094420142</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>38.59920649593993</v>
+        <v>26.10419623332139</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>1.475752415887216</v>
+        <v>0.5619937666619337</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L32" s="2" t="n">
         <v>0</v>
@@ -2168,31 +2168,31 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>4.606444194655385</v>
+        <v>0.038093341404632</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, mfi_strong, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive, foreign_buy_3d, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>6869</v>
+        <v>7799</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>雲豹能源</t>
+          <t>禾榮科</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
         <v/>
       </c>
       <c r="D33" s="2" t="n">
-        <v>606.663640477753</v>
+        <v>611.7499454937273</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>71.2</v>
+        <v>435.5</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -2203,16 +2203,16 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>38.86067094420142</v>
+        <v>60.12411481233664</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>26.10419623332139</v>
+        <v>38.59920649593993</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>0.5619937666619337</v>
+        <v>1.475752415887216</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L33" s="2" t="n">
         <v>0</v>
@@ -2221,11 +2221,11 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>0.038093341404632</v>
+        <v>4.606444194655385</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive, foreign_buy_3d, adx_trending, stronger_than_market</t>
+          <t>rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -2655,21 +2655,21 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>6944</v>
+        <v>6870</v>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>兆聯實業</t>
+          <t>騰雲</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
         <v/>
       </c>
       <c r="D42" s="2" t="n">
-        <v>518.5894468604549</v>
+        <v>518.5352456195039</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>998</v>
+        <v>289</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -2680,16 +2680,16 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>53.97414304544137</v>
+        <v>54.18808299369103</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>13.54217250930741</v>
+        <v>20.69329594231462</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>0.9308369947680232</v>
+        <v>0.1832728974954264</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L42" s="2" t="n">
         <v>0</v>
@@ -2698,31 +2698,31 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>-6.063096853992935</v>
+        <v>-0.7414892129802908</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, kd_golden_cross, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>6870</v>
+        <v>6902</v>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>騰雲</t>
+          <t>GOGOLOOK</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
         <v/>
       </c>
       <c r="D43" s="2" t="n">
-        <v>518.5352456195039</v>
+        <v>508.7113474025167</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>289</v>
+        <v>137.5</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -2733,16 +2733,16 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>54.18808299369103</v>
+        <v>55.36736361158736</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>20.69329594231462</v>
+        <v>20.10381370154674</v>
       </c>
       <c r="J43" s="2" t="n">
-        <v>0.1832728974954264</v>
+        <v>0.2329276147208781</v>
       </c>
       <c r="K43" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L43" s="2" t="n">
         <v>0</v>
@@ -2751,31 +2751,31 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>-0.7414892129802908</v>
+        <v>-0.3703481322627091</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>6916</v>
+        <v>7770</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>華凌</t>
+          <t>君曜</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>513.6132347063674</v>
+        <v>492.5192228975166</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>20.15</v>
+        <v>42.6</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -2786,13 +2786,13 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>49.45269420994582</v>
+        <v>49.23205470173506</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>18.77870919338771</v>
+        <v>6.990383305089063</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>0.212716101588165</v>
+        <v>0.3272373250852448</v>
       </c>
       <c r="K44" s="2" t="n">
         <v>0</v>
@@ -2804,31 +2804,31 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>-0.1541319074217235</v>
+        <v>0.1931446192736043</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>6951</v>
+        <v>7753</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>青新-創</t>
+          <t>星亞</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>509.1065317235509</v>
+        <v>487.9967932480413</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>78.7</v>
+        <v>42.5</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -2839,16 +2839,16 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>47.44109769981664</v>
+        <v>49.18736334439472</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>21.92213186425082</v>
+        <v>25.08255245343453</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>1.246109337475753</v>
+        <v>0.2660209729607627</v>
       </c>
       <c r="K45" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L45" s="2" t="n">
         <v>0</v>
@@ -2857,31 +2857,31 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>0.1838906479945109</v>
+        <v>-0.009245602312927001</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>6902</v>
+        <v>6903</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>GOGOLOOK</t>
+          <t>巨漢</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
         <v/>
       </c>
       <c r="D46" s="2" t="n">
-        <v>508.7113474025167</v>
+        <v>485.3920352556953</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>137.5</v>
+        <v>394</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -2892,13 +2892,13 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>55.36736361158736</v>
+        <v>51.64959307743278</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>20.10381370154674</v>
+        <v>9.970553252553394</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>0.2329276147208781</v>
+        <v>1.369092394743471</v>
       </c>
       <c r="K46" s="2" t="n">
         <v>1</v>
@@ -2910,31 +2910,31 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>-0.3703481322627091</v>
+        <v>-0.2292449030543601</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, williams_r_recovery, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>7770</v>
+        <v>7842</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>君曜</t>
+          <t>天能綠電</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>492.5192228975166</v>
+        <v>480.8956004829969</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>42.6</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2945,16 +2945,16 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>49.23205470173506</v>
+        <v>39.15241912954303</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>6.990383305089063</v>
+        <v>20.35499744177083</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>0.3272373250852448</v>
+        <v>0.187849824274318</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L47" s="2" t="n">
         <v>0</v>
@@ -2963,31 +2963,31 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>0.1931446192736043</v>
+        <v>0.9166581057404332</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>7753</v>
+        <v>7821</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>星亞</t>
+          <t>神數</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>487.9967932480413</v>
+        <v>479.9200867577227</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>42.5</v>
+        <v>41</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2998,16 +2998,16 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>49.18736334439472</v>
+        <v>34.1066205944374</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>25.08255245343453</v>
+        <v>26.67316488192231</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>0.2660209729607627</v>
+        <v>0.3955972118325168</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L48" s="2" t="n">
         <v>0</v>
@@ -3016,31 +3016,31 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>-0.009245602312927001</v>
+        <v>-0.0368639804291439</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>6933</v>
+        <v>6944</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>AMAX-KY</t>
+          <t>兆聯實業</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
         <v/>
       </c>
       <c r="D49" s="2" t="n">
-        <v>487.1411986314473</v>
+        <v>478.589446860455</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>157.5</v>
+        <v>998</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -3051,16 +3051,16 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>53.73800873279094</v>
+        <v>53.97414304544137</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>18.85947881446384</v>
+        <v>13.54217250930741</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>0.9511992847274796</v>
+        <v>0.9308369947680232</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L49" s="2" t="n">
         <v>0</v>
@@ -3069,31 +3069,31 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>1.07590935319981</v>
+        <v>-6.063096853992935</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>breakout_20d, market_above_ma60, avoid_chase, stronger_than_market, cci_momentum, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, kd_golden_cross, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>6903</v>
+        <v>8043</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>巨漢</t>
+          <t>蜜望實</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>485.3920352556953</v>
+        <v>475.7514469076053</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>394</v>
+        <v>173</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -3104,16 +3104,16 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>51.64959307743278</v>
+        <v>46.70045581300656</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>9.970553252553394</v>
+        <v>26.68826088461669</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>1.369092394743471</v>
+        <v>0.402376190359628</v>
       </c>
       <c r="K50" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L50" s="2" t="n">
         <v>0</v>
@@ -3122,31 +3122,31 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-0.2292449030543601</v>
+        <v>-6.202201158697672</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, williams_r_recovery, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>7842</v>
+        <v>6916</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>天能綠電</t>
+          <t>華凌</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>480.8956004829969</v>
+        <v>473.6132347063673</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>97.40000000000001</v>
+        <v>20.15</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -3157,16 +3157,16 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>39.15241912954303</v>
+        <v>49.45269420994582</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>20.35499744177083</v>
+        <v>18.77870919338771</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>0.187849824274318</v>
+        <v>0.212716101588165</v>
       </c>
       <c r="K51" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L51" s="2" t="n">
         <v>0</v>
@@ -3175,31 +3175,31 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>0.9166581057404332</v>
+        <v>-0.1541319074217235</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>7821</v>
+        <v>6951</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>神數</t>
+          <t>青新-創</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>479.9200867577227</v>
+        <v>469.1065317235509</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>41</v>
+        <v>78.7</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -3210,16 +3210,16 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>34.1066205944374</v>
+        <v>47.44109769981664</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>26.67316488192231</v>
+        <v>21.92213186425082</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>0.3955972118325168</v>
+        <v>1.246109337475753</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L52" s="2" t="n">
         <v>0</v>
@@ -3228,31 +3228,31 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>-0.0368639804291439</v>
+        <v>0.1838906479945109</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>8043</v>
+        <v>7744</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>蜜望實</t>
+          <t>崴寶</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>475.7514469076053</v>
+        <v>452.2739161503841</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>173</v>
+        <v>463</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -3263,13 +3263,13 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>46.70045581300656</v>
+        <v>46.63510099871355</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>26.68826088461669</v>
+        <v>12.94767390585702</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>0.402376190359628</v>
+        <v>0.2186238196630761</v>
       </c>
       <c r="K53" s="2" t="n">
         <v>0</v>
@@ -3281,31 +3281,31 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>-6.202201158697672</v>
+        <v>2.634616974798769</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>6924</v>
+        <v>7711</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>榮惠-KY創</t>
+          <t>永擎</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>465.2868228989308</v>
+        <v>448.168402592468</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>130</v>
+        <v>307.5</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -3316,16 +3316,16 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>51.38843437281255</v>
+        <v>33.58404498228191</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>16.82560710356251</v>
+        <v>23.32559148373669</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>1.082274986195472</v>
+        <v>0.3173966296746351</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L54" s="2" t="n">
         <v>0</v>
@@ -3334,31 +3334,31 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.9410840027423416</v>
+        <v>-2.214144684909884</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>7744</v>
+        <v>6933</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>崴寶</t>
+          <t>AMAX-KY</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>452.2739161503841</v>
+        <v>447.1411986314473</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>463</v>
+        <v>157.5</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -3369,13 +3369,13 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>46.63510099871355</v>
+        <v>53.73800873279094</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>12.94767390585702</v>
+        <v>18.85947881446384</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>0.2186238196630761</v>
+        <v>0.9511992847274796</v>
       </c>
       <c r="K55" s="2" t="n">
         <v>0</v>
@@ -3387,31 +3387,31 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>2.634616974798769</v>
+        <v>1.07590935319981</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend</t>
+          <t>breakout_20d, market_above_ma60, avoid_chase, stronger_than_market, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>7711</v>
+        <v>6924</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>永擎</t>
+          <t>榮惠-KY創</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>448.168402592468</v>
+        <v>445.2868228989308</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>307.5</v>
+        <v>130</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -3422,16 +3422,16 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>33.58404498228191</v>
+        <v>51.38843437281255</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>23.32559148373669</v>
+        <v>16.82560710356251</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>0.3173966296746351</v>
+        <v>1.082274986195472</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L56" s="2" t="n">
         <v>0</v>
@@ -3440,11 +3440,11 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>-2.214144684909884</v>
+        <v>0.9410840027423416</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
@@ -4351,21 +4351,21 @@
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>6923</v>
+        <v>6873</v>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>中台</t>
+          <t>泓德能源</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>371.4682919561231</v>
+        <v>375.1231478298613</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>75.40000000000001</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -4376,13 +4376,13 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>44.57626905084211</v>
+        <v>52.88983667921317</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>12.67822019372631</v>
+        <v>15.53961611986994</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>0.8082727665262706</v>
+        <v>0.569297001249601</v>
       </c>
       <c r="K74" s="2" t="n">
         <v>0</v>
@@ -4394,31 +4394,31 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>0.2577025328151188</v>
+        <v>1.068271818973007</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend</t>
+          <t>market_above_ma60, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>7734</v>
+        <v>6862</v>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>印能科技</t>
+          <t>三集瑞-KY</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>370.4252442852194</v>
+        <v>375.0694609867115</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>2835</v>
+        <v>181.5</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -4429,16 +4429,16 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>41.8126328774763</v>
+        <v>44.44859699964978</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>15.66271258074686</v>
+        <v>18.98089112724713</v>
       </c>
       <c r="J75" s="2" t="n">
-        <v>0.2576035571302245</v>
+        <v>0.3280607157287171</v>
       </c>
       <c r="K75" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L75" s="2" t="n">
         <v>0</v>
@@ -4447,31 +4447,31 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-41.22411777427128</v>
+        <v>-2.812789303812949</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>6863</v>
+        <v>7734</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>永道-KY</t>
+          <t>印能科技</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>370.0321392910109</v>
+        <v>370.4252442852194</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>92.8</v>
+        <v>2835</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -4482,16 +4482,16 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>41.40054904091114</v>
+        <v>41.8126328774763</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>20.6022182794955</v>
+        <v>15.66271258074686</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>0.1941587514346871</v>
+        <v>0.2576035571302245</v>
       </c>
       <c r="K76" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L76" s="2" t="n">
         <v>0</v>
@@ -4500,11 +4500,11 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>0.3684407432840513</v>
+        <v>-41.22411777427128</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d</t>
         </is>
       </c>
     </row>
@@ -4563,21 +4563,21 @@
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>6937</v>
+        <v>6971</v>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>天虹</t>
+          <t>惠民實業</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>365.7484381391925</v>
+        <v>363.7964353379251</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>258.5</v>
+        <v>27.3</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
@@ -4588,16 +4588,16 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>41.58821044298968</v>
+        <v>45.75591484800266</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>11.66045158694848</v>
+        <v>18.54081073089325</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>0.5558910775457436</v>
+        <v>0.1202245018776939</v>
       </c>
       <c r="K78" s="2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="L78" s="2" t="n">
         <v>0</v>
@@ -4606,31 +4606,31 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-0.2642627748224893</v>
+        <v>-0.0453578304074157</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, stronger_than_market, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>6971</v>
+        <v>6877</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>惠民實業</t>
+          <t>鏵友益</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>363.7964353379251</v>
+        <v>363.3623638600944</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>27.3</v>
+        <v>132.5</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
@@ -4641,16 +4641,16 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>45.75591484800266</v>
+        <v>47.05222303674569</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>18.54081073089325</v>
+        <v>14.81593521141948</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>0.1202245018776939</v>
+        <v>0.305062344974368</v>
       </c>
       <c r="K79" s="2" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="L79" s="2" t="n">
         <v>0</v>
@@ -4659,31 +4659,31 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>-0.0453578304074157</v>
+        <v>1.002289235069908</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, stronger_than_market, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>6877</v>
+        <v>6936</v>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>鏵友益</t>
+          <t>永鴻生技</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>363.3623638600944</v>
+        <v>360.5870156353577</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>132.5</v>
+        <v>32.65</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
@@ -4694,13 +4694,13 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>47.05222303674569</v>
+        <v>42.20126496160968</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>14.81593521141948</v>
+        <v>13.17221900359745</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>0.305062344974368</v>
+        <v>4.046462224784912</v>
       </c>
       <c r="K80" s="2" t="n">
         <v>2</v>
@@ -4712,31 +4712,31 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>1.002289235069908</v>
+        <v>0.0428852394046692</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>6936</v>
+        <v>7747</v>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>永鴻生技</t>
+          <t>昕奇雲端</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>360.5870156353577</v>
+        <v>359.7446520819408</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>32.65</v>
+        <v>129</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -4747,16 +4747,16 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>42.20126496160968</v>
+        <v>51.76962879405791</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>13.17221900359745</v>
+        <v>4.196623507404667</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>4.046462224784912</v>
+        <v>0.2290081313536389</v>
       </c>
       <c r="K81" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L81" s="2" t="n">
         <v>0</v>
@@ -4765,31 +4765,31 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>0.0428852394046692</v>
+        <v>-0.1267747152922331</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>7747</v>
+        <v>6983</v>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>昕奇雲端</t>
+          <t>華洋精機</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>359.7446520819408</v>
+        <v>358.0912332595235</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>129</v>
+        <v>349.5</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
@@ -4800,13 +4800,13 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>51.76962879405791</v>
+        <v>44.35696361357847</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>4.196623507404667</v>
+        <v>10.04619420799603</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>0.2290081313536389</v>
+        <v>0.3081349841485361</v>
       </c>
       <c r="K82" s="2" t="n">
         <v>0</v>
@@ -4818,31 +4818,31 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>-0.1267747152922331</v>
+        <v>0.69084471980422</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>6983</v>
+        <v>7740</v>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>華洋精機</t>
+          <t>熙特爾-創</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>358.0912332595235</v>
+        <v>357.9738466243005</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>349.5</v>
+        <v>147.5</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
@@ -4853,16 +4853,16 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>44.35696361357847</v>
+        <v>40.20243596528031</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>10.04619420799603</v>
+        <v>19.02230141015969</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>0.3081349841485361</v>
+        <v>0.5163316295136018</v>
       </c>
       <c r="K83" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L83" s="2" t="n">
         <v>0</v>
@@ -4871,31 +4871,31 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>0.69084471980422</v>
+        <v>-0.2294428513595576</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>7740</v>
+        <v>7765</v>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>熙特爾-創</t>
+          <t>中華資安</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>357.9738466243005</v>
+        <v>356.3177662010121</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>147.5</v>
+        <v>221.5</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
@@ -4906,16 +4906,16 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>40.20243596528031</v>
+        <v>38.25188507101979</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>19.02230141015969</v>
+        <v>20.95841076203018</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>0.5163316295136018</v>
+        <v>0.4169676386477593</v>
       </c>
       <c r="K84" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L84" s="2" t="n">
         <v>0</v>
@@ -4924,31 +4924,31 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-0.2294428513595576</v>
+        <v>-0.2425739004286047</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, stronger_than_market</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>7765</v>
+        <v>6914</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>中華資安</t>
+          <t>阜爾運通</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>356.3177662010121</v>
+        <v>351.6461908947728</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>221.5</v>
+        <v>142.5</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
@@ -4959,16 +4959,16 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>38.25188507101979</v>
+        <v>46.91513569723856</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>20.95841076203018</v>
+        <v>9.301055141744916</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>0.4169676386477593</v>
+        <v>0.6707749528069579</v>
       </c>
       <c r="K85" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L85" s="2" t="n">
         <v>0</v>
@@ -4977,31 +4977,31 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-0.2425739004286047</v>
+        <v>0.06783348748948009</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>6873</v>
+        <v>7704</v>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>泓德能源</t>
+          <t>明遠精密</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>355.1231478298612</v>
+        <v>345.9775013456459</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>86.59999999999999</v>
+        <v>60</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
@@ -5012,13 +5012,13 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>52.88983667921317</v>
+        <v>43.08052754930262</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>15.53961611986994</v>
+        <v>10.35003673546126</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>0.569297001249601</v>
+        <v>0.4674774304936214</v>
       </c>
       <c r="K86" s="2" t="n">
         <v>0</v>
@@ -5030,31 +5030,31 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>1.068271818973007</v>
+        <v>-0.2137068832335129</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>6914</v>
+        <v>7792</v>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>阜爾運通</t>
+          <t>安葆</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>351.6461908947728</v>
+        <v>342.0459665854466</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>142.5</v>
+        <v>235.5</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
@@ -5065,16 +5065,16 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>46.91513569723856</v>
+        <v>33.84481336908068</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>9.301055141744916</v>
+        <v>21.04219704037088</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>0.6707749528069579</v>
+        <v>0.4424815915393387</v>
       </c>
       <c r="K87" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L87" s="2" t="n">
         <v>0</v>
@@ -5083,31 +5083,31 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>0.06783348748948009</v>
+        <v>-1.195066356704928</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>7704</v>
+        <v>6855</v>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>明遠精密</t>
+          <t>數泓科</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>345.9775013456459</v>
+        <v>337.4605930448236</v>
       </c>
       <c r="E88" s="2" t="n">
-        <v>60</v>
+        <v>122</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
@@ -5118,13 +5118,13 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>43.08052754930262</v>
+        <v>52.29651938628686</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>10.35003673546126</v>
+        <v>8.04114534922557</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>0.4674774304936214</v>
+        <v>0.6924604135392959</v>
       </c>
       <c r="K88" s="2" t="n">
         <v>0</v>
@@ -5136,31 +5136,31 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>-0.2137068832335129</v>
+        <v>0.4306449892046662</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>6862</v>
+        <v>7728</v>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>三集瑞-KY</t>
+          <t>光焱科技</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>345.0694609867115</v>
+        <v>332.3704498635813</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>181.5</v>
+        <v>654</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
@@ -5171,16 +5171,16 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>44.44859699964978</v>
+        <v>42.17218319386206</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>18.98089112724713</v>
+        <v>11.88058741850058</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>0.3280607157287171</v>
+        <v>0.2558557370213209</v>
       </c>
       <c r="K89" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L89" s="2" t="n">
         <v>0</v>
@@ -5189,31 +5189,31 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-2.812789303812949</v>
+        <v>-2.451909478079361</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>7792</v>
+        <v>6923</v>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>安葆</t>
+          <t>中台</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>342.0459665854466</v>
+        <v>331.4682919561231</v>
       </c>
       <c r="E90" s="2" t="n">
-        <v>235.5</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
@@ -5224,13 +5224,13 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>33.84481336908068</v>
+        <v>44.57626905084211</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>21.04219704037088</v>
+        <v>12.67822019372631</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>0.4424815915393387</v>
+        <v>0.8082727665262706</v>
       </c>
       <c r="K90" s="2" t="n">
         <v>0</v>
@@ -5242,31 +5242,31 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>-1.195066356704928</v>
+        <v>0.2577025328151188</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>6855</v>
+        <v>6863</v>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>數泓科</t>
+          <t>永道-KY</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>337.4605930448236</v>
+        <v>330.0321392910109</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>122</v>
+        <v>92.8</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
@@ -5277,16 +5277,16 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>52.29651938628686</v>
+        <v>41.40054904091114</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>8.04114534922557</v>
+        <v>20.6022182794955</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>0.6924604135392959</v>
+        <v>0.1941587514346871</v>
       </c>
       <c r="K91" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L91" s="2" t="n">
         <v>0</v>
@@ -5295,31 +5295,31 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>0.4306449892046662</v>
+        <v>0.3684407432840513</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>7728</v>
+        <v>6937</v>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>光焱科技</t>
+          <t>天虹</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>332.3704498635813</v>
+        <v>325.7484381391925</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>654</v>
+        <v>258.5</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
@@ -5330,16 +5330,16 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>42.17218319386206</v>
+        <v>41.58821044298968</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>11.88058741850058</v>
+        <v>11.66045158694848</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>0.2558557370213209</v>
+        <v>0.5558910775457436</v>
       </c>
       <c r="K92" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L92" s="2" t="n">
         <v>0</v>
@@ -5348,31 +5348,31 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-2.451909478079361</v>
+        <v>-0.2642627748224893</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>6887</v>
+        <v>7751</v>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>寶綠特-KY</t>
+          <t>竑騰</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>328.9710633676277</v>
+        <v>324.4173100399416</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>33.8</v>
+        <v>1295</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -5383,16 +5383,16 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>45.48886169883458</v>
+        <v>39.44757102375637</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>5.139339190518846</v>
+        <v>9.860766948779018</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>0.6399454679385927</v>
+        <v>1.476844180607912</v>
       </c>
       <c r="K93" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L93" s="2" t="n">
         <v>0</v>
@@ -5401,31 +5401,31 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-0.1638936681527898</v>
+        <v>8.145777824020414</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>7751</v>
+        <v>8047</v>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>竑騰</t>
+          <t>星雲</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>324.4173100399416</v>
+        <v>322.5700999515211</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>1295</v>
+        <v>44</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
@@ -5436,16 +5436,16 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>39.44757102375637</v>
+        <v>39.94849770984634</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>9.860766948779018</v>
+        <v>7.110162534599978</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>1.476844180607912</v>
+        <v>0.8073288779987986</v>
       </c>
       <c r="K94" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L94" s="2" t="n">
         <v>0</v>
@@ -5454,31 +5454,31 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>8.145777824020414</v>
+        <v>-0.5620929104613687</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>8047</v>
+        <v>8045</v>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>星雲</t>
+          <t>達運光電</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>322.5700999515211</v>
+        <v>320.8412753222526</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>44</v>
+        <v>58.4</v>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
@@ -5489,13 +5489,13 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>39.94849770984634</v>
+        <v>38.28273749110956</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>7.110162534599978</v>
+        <v>11.24634823146596</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>0.8073288779987986</v>
+        <v>0.7578615350408903</v>
       </c>
       <c r="K95" s="2" t="n">
         <v>1</v>
@@ -5507,31 +5507,31 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-0.5620929104613687</v>
+        <v>0.1666947706218837</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>8045</v>
+        <v>6887</v>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>達運光電</t>
+          <t>寶綠特-KY</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>320.8412753222526</v>
+        <v>308.9710633676277</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>58.4</v>
+        <v>33.8</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -5542,13 +5542,13 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>38.28273749110956</v>
+        <v>45.48886169883458</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>11.24634823146596</v>
+        <v>5.139339190518846</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>0.7578615350408903</v>
+        <v>0.6399454679385927</v>
       </c>
       <c r="K96" s="2" t="n">
         <v>1</v>
@@ -5560,31 +5560,31 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>0.1666947706218837</v>
+        <v>-0.1638936681527898</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>6854</v>
+        <v>7736</v>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>錼創科技-KY創</t>
+          <t>虎山</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>307.9321804976679</v>
+        <v>304.467327106767</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>113.5</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
@@ -5595,16 +5595,16 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>29.76518114133657</v>
+        <v>41.22229868003949</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>23.47971786607372</v>
+        <v>13.28760285875499</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>1.527707214277649</v>
+        <v>0.8334829319487406</v>
       </c>
       <c r="K97" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L97" s="2" t="n">
         <v>0</v>
@@ -5613,31 +5613,31 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-0.1925840124130724</v>
+        <v>0.0114340746977891</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>7736</v>
+        <v>8032</v>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>虎山</t>
+          <t>光菱</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>304.467327106767</v>
+        <v>301.7152547634907</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>70.40000000000001</v>
+        <v>41.8</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5648,16 +5648,16 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>41.22229868003949</v>
+        <v>41.29813014855965</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>13.28760285875499</v>
+        <v>19.24859766789432</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>0.8334829319487406</v>
+        <v>0.1251730459362888</v>
       </c>
       <c r="K98" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L98" s="2" t="n">
         <v>0</v>
@@ -5666,31 +5666,31 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>0.0114340746977891</v>
+        <v>-0.4744961205503365</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>8032</v>
+        <v>6906</v>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>光菱</t>
+          <t>現觀科</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
         <v/>
       </c>
       <c r="D99" s="2" t="n">
-        <v>301.7152547634907</v>
+        <v>298.577190325238</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>41.8</v>
+        <v>82</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
@@ -5701,16 +5701,16 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>41.29813014855965</v>
+        <v>39.51278555185927</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>19.24859766789432</v>
+        <v>17.85269472786651</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>0.1251730459362888</v>
+        <v>0.3971803849544118</v>
       </c>
       <c r="K99" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L99" s="2" t="n">
         <v>0</v>
@@ -5719,7 +5719,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-0.4744961205503365</v>
+        <v>-1.468828733260629</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5729,21 +5729,21 @@
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>6906</v>
+        <v>6918</v>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>現觀科</t>
+          <t>愛派司</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>298.577190325238</v>
+        <v>297.0850751975527</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>82</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
@@ -5754,13 +5754,13 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>39.51278555185927</v>
+        <v>52.23885075978043</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>17.85269472786651</v>
+        <v>13.4830962017074</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>0.3971803849544118</v>
+        <v>0.4409605856337868</v>
       </c>
       <c r="K100" s="2" t="n">
         <v>1</v>
@@ -5772,31 +5772,31 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-1.468828733260629</v>
+        <v>0.1896822961093553</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
-        <v>6918</v>
+        <v>6931</v>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>愛派司</t>
+          <t>青松健康</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>297.0850751975527</v>
+        <v>296.6313441542502</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>74.09999999999999</v>
+        <v>39.75</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
@@ -5807,13 +5807,13 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>52.23885075978043</v>
+        <v>40.62086957529913</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>13.4830962017074</v>
+        <v>17.3503840018668</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>0.4409605856337868</v>
+        <v>0.5679778257363548</v>
       </c>
       <c r="K101" s="2" t="n">
         <v>1</v>
@@ -5825,7 +5825,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>0.1896822961093553</v>
+        <v>0.068982221357753</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5835,21 +5835,21 @@
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
-        <v>6931</v>
+        <v>7721</v>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>青松健康</t>
+          <t>微程式</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>296.6313441542502</v>
+        <v>294.8380842922334</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>39.75</v>
+        <v>71</v>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
@@ -5860,16 +5860,16 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>40.62086957529913</v>
+        <v>44.80168470812589</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>17.3503840018668</v>
+        <v>10.93154352012251</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>0.5679778257363548</v>
+        <v>0.1445584497526122</v>
       </c>
       <c r="K102" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L102" s="2" t="n">
         <v>0</v>
@@ -5878,31 +5878,31 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>0.068982221357753</v>
+        <v>-0.2848709066211199</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
-        <v>7721</v>
+        <v>6967</v>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>微程式</t>
+          <t>汎瑋材料</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>294.8380842922334</v>
+        <v>294.6658513074201</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>71</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
@@ -5913,13 +5913,13 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>44.80168470812589</v>
+        <v>43.2632513968686</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>10.93154352012251</v>
+        <v>12.28915740397964</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>0.1445584497526122</v>
+        <v>0.6501533329938837</v>
       </c>
       <c r="K103" s="2" t="n">
         <v>0</v>
@@ -5931,31 +5931,31 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-0.2848709066211199</v>
+        <v>-0.1277832835988867</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
-        <v>6967</v>
+        <v>6854</v>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>汎瑋材料</t>
+          <t>錼創科技-KY創</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>294.6658513074201</v>
+        <v>287.9321804976679</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>69.40000000000001</v>
+        <v>113.5</v>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
@@ -5966,13 +5966,13 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>43.2632513968686</v>
+        <v>29.76518114133657</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>12.28915740397964</v>
+        <v>23.47971786607372</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>0.6501533329938837</v>
+        <v>1.527707214277649</v>
       </c>
       <c r="K104" s="2" t="n">
         <v>0</v>
@@ -5984,11 +5984,11 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-0.1277832835988867</v>
+        <v>-0.1925840124130724</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
@@ -6418,21 +6418,21 @@
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
-        <v>6909</v>
+        <v>6908</v>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>創控</t>
+          <t>宏碁遊戲-創</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>257.2207977387619</v>
+        <v>243.6464737414201</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>51.3</v>
+        <v>36.6</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
@@ -6443,13 +6443,13 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>44.84173236254644</v>
+        <v>35.67848240626194</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>16.43522249029083</v>
+        <v>16.1613569677956</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>0.2418643455155242</v>
+        <v>0.9148933175702304</v>
       </c>
       <c r="K113" s="2" t="n">
         <v>0</v>
@@ -6461,11 +6461,11 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-0.4028328879516456</v>
+        <v>-0.08735674367619881</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
@@ -6630,21 +6630,21 @@
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
-        <v>6899</v>
+        <v>6921</v>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>創為精密</t>
+          <t>嘉雨思-創</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
         <v/>
       </c>
       <c r="D117" s="2" t="n">
-        <v>218.6683684623978</v>
+        <v>226.6310574268157</v>
       </c>
       <c r="E117" s="2" t="n">
-        <v>54.7</v>
+        <v>68</v>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
@@ -6655,13 +6655,13 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>34.04625825395961</v>
+        <v>38.93343411596706</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>14.93820479383245</v>
+        <v>17.35227948019281</v>
       </c>
       <c r="J117" s="2" t="n">
-        <v>0.9242118449439766</v>
+        <v>0.1668720314980874</v>
       </c>
       <c r="K117" s="2" t="n">
         <v>0</v>
@@ -6673,31 +6673,31 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-0.3323764673576509</v>
+        <v>0.2385507695230706</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
-        <v>7749</v>
+        <v>6899</v>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>意騰-KY</t>
+          <t>創為精密</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>216.15866189966</v>
+        <v>218.6683684623978</v>
       </c>
       <c r="E118" s="2" t="n">
-        <v>404</v>
+        <v>54.7</v>
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
@@ -6708,13 +6708,13 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>34.08472250739553</v>
+        <v>34.04625825395961</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>15.49490569347116</v>
+        <v>14.93820479383245</v>
       </c>
       <c r="J118" s="2" t="n">
-        <v>0.2834734020563929</v>
+        <v>0.9242118449439766</v>
       </c>
       <c r="K118" s="2" t="n">
         <v>0</v>
@@ -6726,31 +6726,31 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>-4.924311626850146</v>
+        <v>-0.3323764673576509</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
-        <v>6885</v>
+        <v>6909</v>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>全福生技</t>
+          <t>創控</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>215.2736476833169</v>
+        <v>217.220797738762</v>
       </c>
       <c r="E119" s="2" t="n">
-        <v>21.85</v>
+        <v>51.3</v>
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
@@ -6761,16 +6761,16 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>47.2964484181453</v>
+        <v>44.84173236254644</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>17.69471854733938</v>
+        <v>16.43522249029083</v>
       </c>
       <c r="J119" s="2" t="n">
-        <v>0.4064297818704699</v>
+        <v>0.2418643455155242</v>
       </c>
       <c r="K119" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L119" s="2" t="n">
         <v>0</v>
@@ -6779,31 +6779,31 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>0.06826108265377059</v>
+        <v>-0.4028328879516456</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
-        <v>8044</v>
+        <v>7749</v>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>網家</t>
+          <t>意騰-KY</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>214.1764594044797</v>
+        <v>216.15866189966</v>
       </c>
       <c r="E120" s="2" t="n">
-        <v>26.8</v>
+        <v>404</v>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
@@ -6814,13 +6814,13 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>41.52098254858291</v>
+        <v>34.08472250739553</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>14.18891225190132</v>
+        <v>15.49490569347116</v>
       </c>
       <c r="J120" s="2" t="n">
-        <v>0.2486213192443414</v>
+        <v>0.2834734020563929</v>
       </c>
       <c r="K120" s="2" t="n">
         <v>0</v>
@@ -6832,31 +6832,31 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-0.3977575223101354</v>
+        <v>-4.924311626850146</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
-        <v>6908</v>
+        <v>6885</v>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>宏碁遊戲-創</t>
+          <t>全福生技</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
         <v/>
       </c>
       <c r="D121" s="2" t="n">
-        <v>213.6464737414201</v>
+        <v>215.2736476833169</v>
       </c>
       <c r="E121" s="2" t="n">
-        <v>36.6</v>
+        <v>21.85</v>
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
@@ -6867,16 +6867,16 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>35.67848240626194</v>
+        <v>47.2964484181453</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>16.1613569677956</v>
+        <v>17.69471854733938</v>
       </c>
       <c r="J121" s="2" t="n">
-        <v>0.9148933175702304</v>
+        <v>0.4064297818704699</v>
       </c>
       <c r="K121" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L121" s="2" t="n">
         <v>0</v>
@@ -6885,7 +6885,7 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>-0.08735674367619881</v>
+        <v>0.06826108265377059</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
@@ -6895,21 +6895,21 @@
     </row>
     <row r="122">
       <c r="A122" s="2" t="n">
-        <v>7730</v>
+        <v>8044</v>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>暉盛-創</t>
+          <t>網家</t>
         </is>
       </c>
       <c r="C122" s="2" t="n">
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>209.1135777707526</v>
+        <v>214.1764594044797</v>
       </c>
       <c r="E122" s="2" t="n">
-        <v>183</v>
+        <v>26.8</v>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
@@ -6920,13 +6920,13 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>47.84907312567253</v>
+        <v>41.52098254858291</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>10.27348699793313</v>
+        <v>14.18891225190132</v>
       </c>
       <c r="J122" s="2" t="n">
-        <v>0.9215102340619056</v>
+        <v>0.2486213192443414</v>
       </c>
       <c r="K122" s="2" t="n">
         <v>0</v>
@@ -6938,31 +6938,31 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>0.4485259988977426</v>
+        <v>-0.3977575223101354</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="n">
-        <v>6953</v>
+        <v>7730</v>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>家碩</t>
+          <t>暉盛-創</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
         <v/>
       </c>
       <c r="D123" s="2" t="n">
-        <v>202.7766110895432</v>
+        <v>209.1135777707526</v>
       </c>
       <c r="E123" s="2" t="n">
-        <v>228</v>
+        <v>183</v>
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
@@ -6973,13 +6973,13 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>43.79332010999956</v>
+        <v>47.84907312567253</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>12.77746564868914</v>
+        <v>10.27348699793313</v>
       </c>
       <c r="J123" s="2" t="n">
-        <v>0.3861295447556247</v>
+        <v>0.9215102340619056</v>
       </c>
       <c r="K123" s="2" t="n">
         <v>0</v>
@@ -6991,7 +6991,7 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>0.2059930994131873</v>
+        <v>0.4485259988977426</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
@@ -7001,21 +7001,21 @@
     </row>
     <row r="124">
       <c r="A124" s="2" t="n">
-        <v>6859</v>
+        <v>6953</v>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>伯特光</t>
+          <t>家碩</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
         <v/>
       </c>
       <c r="D124" s="2" t="n">
-        <v>202.4637793579379</v>
+        <v>202.7766110895432</v>
       </c>
       <c r="E124" s="2" t="n">
-        <v>120.5</v>
+        <v>228</v>
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
@@ -7026,13 +7026,13 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>42.96529548176591</v>
+        <v>43.79332010999956</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>15.9452175682549</v>
+        <v>12.77746564868914</v>
       </c>
       <c r="J124" s="2" t="n">
-        <v>0.1066902570738212</v>
+        <v>0.3861295447556247</v>
       </c>
       <c r="K124" s="2" t="n">
         <v>0</v>
@@ -7044,31 +7044,31 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>-1.061681770343376</v>
+        <v>0.2059930994131873</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, dealer_buy_3d</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="n">
-        <v>6921</v>
+        <v>6859</v>
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>嘉雨思-創</t>
+          <t>伯特光</t>
         </is>
       </c>
       <c r="C125" s="2" t="n">
         <v/>
       </c>
       <c r="D125" s="2" t="n">
-        <v>196.6310574268157</v>
+        <v>202.4637793579379</v>
       </c>
       <c r="E125" s="2" t="n">
-        <v>68</v>
+        <v>120.5</v>
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
@@ -7079,13 +7079,13 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>38.93343411596706</v>
+        <v>42.96529548176591</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>17.35227948019281</v>
+        <v>15.9452175682549</v>
       </c>
       <c r="J125" s="2" t="n">
-        <v>0.1668720314980874</v>
+        <v>0.1066902570738212</v>
       </c>
       <c r="K125" s="2" t="n">
         <v>0</v>
@@ -7097,11 +7097,11 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>0.2385507695230706</v>
+        <v>-1.061681770343376</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, dealer_buy_3d</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
scan: seg7 2026-07-10 18:49 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq8_2026-07-09.xlsx
+++ b/output/full_scan/batch_seq8_2026-07-09.xlsx
@@ -1754,21 +1754,21 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>7402</v>
+        <v>6928</v>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>邑錡</t>
+          <t>攸泰科技</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
         <v/>
       </c>
       <c r="D25" s="2" t="n">
-        <v>657.9599836910082</v>
+        <v>660.356434821952</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>131</v>
+        <v>53.3</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
@@ -1779,13 +1779,13 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>63.74607051890244</v>
+        <v>57.63566193007057</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>31.87193742892348</v>
+        <v>32.03870086834914</v>
       </c>
       <c r="J25" s="2" t="n">
-        <v>1.895998369100822</v>
+        <v>0.4347882539286762</v>
       </c>
       <c r="K25" s="2" t="n">
         <v>0</v>
@@ -1797,31 +1797,31 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>3.251686895042466</v>
+        <v>0.3178441433848018</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>volume_break, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, mfi_strong, above_ichimoku_cloud</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>6965</v>
+        <v>7402</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>中傑-KY</t>
+          <t>邑錡</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
         <v/>
       </c>
       <c r="D26" s="2" t="n">
-        <v>657.1843931304295</v>
+        <v>657.9599836910082</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>80</v>
+        <v>131</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
@@ -1832,16 +1832,16 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>52.20498622387128</v>
+        <v>63.74607051890244</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>22.25081504807666</v>
+        <v>31.87193742892348</v>
       </c>
       <c r="J26" s="2" t="n">
-        <v>0.5680626029119896</v>
+        <v>1.895998369100822</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L26" s="2" t="n">
         <v>0</v>
@@ -1850,31 +1850,31 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>0.151930499100081</v>
+        <v>3.251686895042466</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>volume_break, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>6890</v>
+        <v>6965</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>來億-KY</t>
+          <t>中傑-KY</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
         <v/>
       </c>
       <c r="D27" s="2" t="n">
-        <v>655.1476617649607</v>
+        <v>657.1843931304295</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>206</v>
+        <v>80</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
@@ -1885,49 +1885,49 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>47.04697220223746</v>
+        <v>52.20498622387128</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>18.8247603452546</v>
+        <v>22.25081504807666</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>0.9427276747293294</v>
+        <v>0.5680626029119896</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M27" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>-4.348860042339972</v>
+        <v>0.151930499100081</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, liquidity_ok, stronger_than_market, kd_golden_cross, obv_uptrend, invest_trust_buy_2d, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>7717</v>
+        <v>6890</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>萊德光電-KY</t>
+          <t>來億-KY</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v/>
       </c>
       <c r="D28" s="2" t="n">
-        <v>652.2429131338725</v>
+        <v>655.1476617649607</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>422.5</v>
+        <v>206</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -1938,49 +1938,49 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>32.03154027332101</v>
+        <v>47.04697220223746</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>22.98215457332702</v>
+        <v>18.8247603452546</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>0.2816613219084758</v>
+        <v>0.9427276747293294</v>
       </c>
       <c r="K28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L28" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M28" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>0.6582596039140114</v>
+        <v>-4.348860042339972</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, hist_turn_positive, adx_trending, stronger_than_market</t>
+          <t>market_above_ma60, liquidity_ok, stronger_than_market, kd_golden_cross, obv_uptrend, invest_trust_buy_2d, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>6928</v>
+        <v>7717</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>攸泰科技</t>
+          <t>萊德光電-KY</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
         <v/>
       </c>
       <c r="D29" s="2" t="n">
-        <v>640.356434821952</v>
+        <v>652.2429131338725</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>53.3</v>
+        <v>422.5</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
@@ -1991,13 +1991,13 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>57.63566193007057</v>
+        <v>32.03154027332101</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>32.03870086834914</v>
+        <v>22.98215457332702</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>0.4347882539286762</v>
+        <v>0.2816613219084758</v>
       </c>
       <c r="K29" s="2" t="n">
         <v>0</v>
@@ -2009,11 +2009,11 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>0.3178441433848018</v>
+        <v>0.6582596039140114</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, hist_turn_positive, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
@@ -2125,21 +2125,21 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>6869</v>
+        <v>7799</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>雲豹能源</t>
+          <t>禾榮科</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>626.663640477753</v>
+        <v>611.7499454937273</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>71.2</v>
+        <v>435.5</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -2150,16 +2150,16 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>38.86067094420142</v>
+        <v>60.12411481233664</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>26.10419623332139</v>
+        <v>38.59920649593993</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>0.5619937666619337</v>
+        <v>1.475752415887216</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L32" s="2" t="n">
         <v>0</v>
@@ -2168,31 +2168,31 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>0.038093341404632</v>
+        <v>4.606444194655385</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive, foreign_buy_3d, adx_trending, stronger_than_market</t>
+          <t>rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>7799</v>
+        <v>6869</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>禾榮科</t>
+          <t>雲豹能源</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
         <v/>
       </c>
       <c r="D33" s="2" t="n">
-        <v>611.7499454937273</v>
+        <v>606.663640477753</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>435.5</v>
+        <v>71.2</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -2203,16 +2203,16 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>60.12411481233664</v>
+        <v>38.86067094420142</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>38.59920649593993</v>
+        <v>26.10419623332139</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>1.475752415887216</v>
+        <v>0.5619937666619337</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L33" s="2" t="n">
         <v>0</v>
@@ -2221,11 +2221,11 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>4.606444194655385</v>
+        <v>0.038093341404632</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, mfi_strong, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive, foreign_buy_3d, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
@@ -2655,21 +2655,21 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>6870</v>
+        <v>6944</v>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>騰雲</t>
+          <t>兆聯實業</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
         <v/>
       </c>
       <c r="D42" s="2" t="n">
-        <v>518.5352456195039</v>
+        <v>518.5894468604549</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>289</v>
+        <v>998</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -2680,16 +2680,16 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>54.18808299369103</v>
+        <v>53.97414304544137</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>20.69329594231462</v>
+        <v>13.54217250930741</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>0.1832728974954264</v>
+        <v>0.9308369947680232</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L42" s="2" t="n">
         <v>0</v>
@@ -2698,31 +2698,31 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>-0.7414892129802908</v>
+        <v>-6.063096853992935</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, kd_golden_cross, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>6902</v>
+        <v>6870</v>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>GOGOLOOK</t>
+          <t>騰雲</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
         <v/>
       </c>
       <c r="D43" s="2" t="n">
-        <v>508.7113474025167</v>
+        <v>518.5352456195039</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>137.5</v>
+        <v>289</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -2733,16 +2733,16 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>55.36736361158736</v>
+        <v>54.18808299369103</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>20.10381370154674</v>
+        <v>20.69329594231462</v>
       </c>
       <c r="J43" s="2" t="n">
-        <v>0.2329276147208781</v>
+        <v>0.1832728974954264</v>
       </c>
       <c r="K43" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L43" s="2" t="n">
         <v>0</v>
@@ -2751,31 +2751,31 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>-0.3703481322627091</v>
+        <v>-0.7414892129802908</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>7770</v>
+        <v>6916</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>君曜</t>
+          <t>華凌</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>492.5192228975166</v>
+        <v>513.6132347063674</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>42.6</v>
+        <v>20.15</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -2786,13 +2786,13 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>49.23205470173506</v>
+        <v>49.45269420994582</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>6.990383305089063</v>
+        <v>18.77870919338771</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>0.3272373250852448</v>
+        <v>0.212716101588165</v>
       </c>
       <c r="K44" s="2" t="n">
         <v>0</v>
@@ -2804,31 +2804,31 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>0.1931446192736043</v>
+        <v>-0.1541319074217235</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>7753</v>
+        <v>6951</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>星亞</t>
+          <t>青新-創</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>487.9967932480413</v>
+        <v>509.1065317235509</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>42.5</v>
+        <v>78.7</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -2839,16 +2839,16 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>49.18736334439472</v>
+        <v>47.44109769981664</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>25.08255245343453</v>
+        <v>21.92213186425082</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>0.2660209729607627</v>
+        <v>1.246109337475753</v>
       </c>
       <c r="K45" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L45" s="2" t="n">
         <v>0</v>
@@ -2857,31 +2857,31 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>-0.009245602312927001</v>
+        <v>0.1838906479945109</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>6903</v>
+        <v>6902</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>巨漢</t>
+          <t>GOGOLOOK</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
         <v/>
       </c>
       <c r="D46" s="2" t="n">
-        <v>485.3920352556953</v>
+        <v>508.7113474025167</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>394</v>
+        <v>137.5</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -2892,13 +2892,13 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>51.64959307743278</v>
+        <v>55.36736361158736</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>9.970553252553394</v>
+        <v>20.10381370154674</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>1.369092394743471</v>
+        <v>0.2329276147208781</v>
       </c>
       <c r="K46" s="2" t="n">
         <v>1</v>
@@ -2910,31 +2910,31 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>-0.2292449030543601</v>
+        <v>-0.3703481322627091</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, williams_r_recovery, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>7842</v>
+        <v>7770</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>天能綠電</t>
+          <t>君曜</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>480.8956004829969</v>
+        <v>492.5192228975166</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>97.40000000000001</v>
+        <v>42.6</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2945,16 +2945,16 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>39.15241912954303</v>
+        <v>49.23205470173506</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>20.35499744177083</v>
+        <v>6.990383305089063</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>0.187849824274318</v>
+        <v>0.3272373250852448</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L47" s="2" t="n">
         <v>0</v>
@@ -2963,31 +2963,31 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>0.9166581057404332</v>
+        <v>0.1931446192736043</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>7821</v>
+        <v>7753</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>神數</t>
+          <t>星亞</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>479.9200867577227</v>
+        <v>487.9967932480413</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>41</v>
+        <v>42.5</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2998,16 +2998,16 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>34.1066205944374</v>
+        <v>49.18736334439472</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>26.67316488192231</v>
+        <v>25.08255245343453</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>0.3955972118325168</v>
+        <v>0.2660209729607627</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L48" s="2" t="n">
         <v>0</v>
@@ -3016,31 +3016,31 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>-0.0368639804291439</v>
+        <v>-0.009245602312927001</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>6944</v>
+        <v>6933</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>兆聯實業</t>
+          <t>AMAX-KY</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
         <v/>
       </c>
       <c r="D49" s="2" t="n">
-        <v>478.589446860455</v>
+        <v>487.1411986314473</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>998</v>
+        <v>157.5</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -3051,16 +3051,16 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>53.97414304544137</v>
+        <v>53.73800873279094</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>13.54217250930741</v>
+        <v>18.85947881446384</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>0.9308369947680232</v>
+        <v>0.9511992847274796</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L49" s="2" t="n">
         <v>0</v>
@@ -3069,31 +3069,31 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>-6.063096853992935</v>
+        <v>1.07590935319981</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, kd_golden_cross, above_ichimoku_cloud</t>
+          <t>breakout_20d, market_above_ma60, avoid_chase, stronger_than_market, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>8043</v>
+        <v>6903</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>蜜望實</t>
+          <t>巨漢</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>475.7514469076053</v>
+        <v>485.3920352556953</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>173</v>
+        <v>394</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -3104,16 +3104,16 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>46.70045581300656</v>
+        <v>51.64959307743278</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>26.68826088461669</v>
+        <v>9.970553252553394</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>0.402376190359628</v>
+        <v>1.369092394743471</v>
       </c>
       <c r="K50" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L50" s="2" t="n">
         <v>0</v>
@@ -3122,31 +3122,31 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-6.202201158697672</v>
+        <v>-0.2292449030543601</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, williams_r_recovery, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>6916</v>
+        <v>7842</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>華凌</t>
+          <t>天能綠電</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>473.6132347063673</v>
+        <v>480.8956004829969</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>20.15</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -3157,16 +3157,16 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>49.45269420994582</v>
+        <v>39.15241912954303</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>18.77870919338771</v>
+        <v>20.35499744177083</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>0.212716101588165</v>
+        <v>0.187849824274318</v>
       </c>
       <c r="K51" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L51" s="2" t="n">
         <v>0</v>
@@ -3175,31 +3175,31 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>-0.1541319074217235</v>
+        <v>0.9166581057404332</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>6951</v>
+        <v>7821</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>青新-創</t>
+          <t>神數</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>469.1065317235509</v>
+        <v>479.9200867577227</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>78.7</v>
+        <v>41</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -3210,16 +3210,16 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>47.44109769981664</v>
+        <v>34.1066205944374</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>21.92213186425082</v>
+        <v>26.67316488192231</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>1.246109337475753</v>
+        <v>0.3955972118325168</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L52" s="2" t="n">
         <v>0</v>
@@ -3228,31 +3228,31 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>0.1838906479945109</v>
+        <v>-0.0368639804291439</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>7744</v>
+        <v>8043</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>崴寶</t>
+          <t>蜜望實</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>452.2739161503841</v>
+        <v>475.7514469076053</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>463</v>
+        <v>173</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -3263,13 +3263,13 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>46.63510099871355</v>
+        <v>46.70045581300656</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>12.94767390585702</v>
+        <v>26.68826088461669</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>0.2186238196630761</v>
+        <v>0.402376190359628</v>
       </c>
       <c r="K53" s="2" t="n">
         <v>0</v>
@@ -3281,31 +3281,31 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>2.634616974798769</v>
+        <v>-6.202201158697672</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>7711</v>
+        <v>6924</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>永擎</t>
+          <t>榮惠-KY創</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>448.168402592468</v>
+        <v>465.2868228989308</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>307.5</v>
+        <v>130</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -3316,16 +3316,16 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>33.58404498228191</v>
+        <v>51.38843437281255</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>23.32559148373669</v>
+        <v>16.82560710356251</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>0.3173966296746351</v>
+        <v>1.082274986195472</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L54" s="2" t="n">
         <v>0</v>
@@ -3334,31 +3334,31 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>-2.214144684909884</v>
+        <v>0.9410840027423416</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>6933</v>
+        <v>7744</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>AMAX-KY</t>
+          <t>崴寶</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>447.1411986314473</v>
+        <v>452.2739161503841</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>157.5</v>
+        <v>463</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -3369,13 +3369,13 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>53.73800873279094</v>
+        <v>46.63510099871355</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>18.85947881446384</v>
+        <v>12.94767390585702</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>0.9511992847274796</v>
+        <v>0.2186238196630761</v>
       </c>
       <c r="K55" s="2" t="n">
         <v>0</v>
@@ -3387,31 +3387,31 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>1.07590935319981</v>
+        <v>2.634616974798769</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>breakout_20d, market_above_ma60, avoid_chase, stronger_than_market, cci_momentum, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>6924</v>
+        <v>7711</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>榮惠-KY創</t>
+          <t>永擎</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>445.2868228989308</v>
+        <v>448.168402592468</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>130</v>
+        <v>307.5</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -3422,16 +3422,16 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>51.38843437281255</v>
+        <v>33.58404498228191</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>16.82560710356251</v>
+        <v>23.32559148373669</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>1.082274986195472</v>
+        <v>0.3173966296746351</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L56" s="2" t="n">
         <v>0</v>
@@ -3440,11 +3440,11 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.9410840027423416</v>
+        <v>-2.214144684909884</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
@@ -4351,21 +4351,21 @@
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>6873</v>
+        <v>6923</v>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>泓德能源</t>
+          <t>中台</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>375.1231478298613</v>
+        <v>371.4682919561231</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>86.59999999999999</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -4376,13 +4376,13 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>52.88983667921317</v>
+        <v>44.57626905084211</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>15.53961611986994</v>
+        <v>12.67822019372631</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>0.569297001249601</v>
+        <v>0.8082727665262706</v>
       </c>
       <c r="K74" s="2" t="n">
         <v>0</v>
@@ -4394,31 +4394,31 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>1.068271818973007</v>
+        <v>0.2577025328151188</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>6862</v>
+        <v>7734</v>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>三集瑞-KY</t>
+          <t>印能科技</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>375.0694609867115</v>
+        <v>370.4252442852194</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>181.5</v>
+        <v>2835</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -4429,16 +4429,16 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>44.44859699964978</v>
+        <v>41.8126328774763</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>18.98089112724713</v>
+        <v>15.66271258074686</v>
       </c>
       <c r="J75" s="2" t="n">
-        <v>0.3280607157287171</v>
+        <v>0.2576035571302245</v>
       </c>
       <c r="K75" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L75" s="2" t="n">
         <v>0</v>
@@ -4447,31 +4447,31 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-2.812789303812949</v>
+        <v>-41.22411777427128</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>7734</v>
+        <v>6863</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>印能科技</t>
+          <t>永道-KY</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>370.4252442852194</v>
+        <v>370.0321392910109</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>2835</v>
+        <v>92.8</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -4482,16 +4482,16 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>41.8126328774763</v>
+        <v>41.40054904091114</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>15.66271258074686</v>
+        <v>20.6022182794955</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>0.2576035571302245</v>
+        <v>0.1941587514346871</v>
       </c>
       <c r="K76" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L76" s="2" t="n">
         <v>0</v>
@@ -4500,11 +4500,11 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-41.22411777427128</v>
+        <v>0.3684407432840513</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
@@ -4563,21 +4563,21 @@
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>6971</v>
+        <v>6937</v>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>惠民實業</t>
+          <t>天虹</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>363.7964353379251</v>
+        <v>365.7484381391925</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>27.3</v>
+        <v>258.5</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
@@ -4588,16 +4588,16 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>45.75591484800266</v>
+        <v>41.58821044298968</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>18.54081073089325</v>
+        <v>11.66045158694848</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>0.1202245018776939</v>
+        <v>0.5558910775457436</v>
       </c>
       <c r="K78" s="2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L78" s="2" t="n">
         <v>0</v>
@@ -4606,31 +4606,31 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-0.0453578304074157</v>
+        <v>-0.2642627748224893</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, stronger_than_market, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>6877</v>
+        <v>6971</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>鏵友益</t>
+          <t>惠民實業</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>363.3623638600944</v>
+        <v>363.7964353379251</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>132.5</v>
+        <v>27.3</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
@@ -4641,16 +4641,16 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>47.05222303674569</v>
+        <v>45.75591484800266</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>14.81593521141948</v>
+        <v>18.54081073089325</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>0.305062344974368</v>
+        <v>0.1202245018776939</v>
       </c>
       <c r="K79" s="2" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="L79" s="2" t="n">
         <v>0</v>
@@ -4659,31 +4659,31 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>1.002289235069908</v>
+        <v>-0.0453578304074157</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, stronger_than_market, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>6936</v>
+        <v>6877</v>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>永鴻生技</t>
+          <t>鏵友益</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>360.5870156353577</v>
+        <v>363.3623638600944</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>32.65</v>
+        <v>132.5</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
@@ -4694,13 +4694,13 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>42.20126496160968</v>
+        <v>47.05222303674569</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>13.17221900359745</v>
+        <v>14.81593521141948</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>4.046462224784912</v>
+        <v>0.305062344974368</v>
       </c>
       <c r="K80" s="2" t="n">
         <v>2</v>
@@ -4712,31 +4712,31 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>0.0428852394046692</v>
+        <v>1.002289235069908</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>7747</v>
+        <v>6936</v>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>昕奇雲端</t>
+          <t>永鴻生技</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>359.7446520819408</v>
+        <v>360.5870156353577</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>129</v>
+        <v>32.65</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -4747,16 +4747,16 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>51.76962879405791</v>
+        <v>42.20126496160968</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>4.196623507404667</v>
+        <v>13.17221900359745</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>0.2290081313536389</v>
+        <v>4.046462224784912</v>
       </c>
       <c r="K81" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L81" s="2" t="n">
         <v>0</v>
@@ -4765,31 +4765,31 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>-0.1267747152922331</v>
+        <v>0.0428852394046692</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong, above_ichimoku_cloud</t>
+          <t>volume_break, market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>6983</v>
+        <v>7747</v>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>華洋精機</t>
+          <t>昕奇雲端</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>358.0912332595235</v>
+        <v>359.7446520819408</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>349.5</v>
+        <v>129</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
@@ -4800,13 +4800,13 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>44.35696361357847</v>
+        <v>51.76962879405791</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>10.04619420799603</v>
+        <v>4.196623507404667</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>0.3081349841485361</v>
+        <v>0.2290081313536389</v>
       </c>
       <c r="K82" s="2" t="n">
         <v>0</v>
@@ -4818,31 +4818,31 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>0.69084471980422</v>
+        <v>-0.1267747152922331</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>7740</v>
+        <v>6983</v>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>熙特爾-創</t>
+          <t>華洋精機</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>357.9738466243005</v>
+        <v>358.0912332595235</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>147.5</v>
+        <v>349.5</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
@@ -4853,16 +4853,16 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>40.20243596528031</v>
+        <v>44.35696361357847</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>19.02230141015969</v>
+        <v>10.04619420799603</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>0.5163316295136018</v>
+        <v>0.3081349841485361</v>
       </c>
       <c r="K83" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L83" s="2" t="n">
         <v>0</v>
@@ -4871,31 +4871,31 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>-0.2294428513595576</v>
+        <v>0.69084471980422</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>7765</v>
+        <v>7740</v>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>中華資安</t>
+          <t>熙特爾-創</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>356.3177662010121</v>
+        <v>357.9738466243005</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>221.5</v>
+        <v>147.5</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
@@ -4906,16 +4906,16 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>38.25188507101979</v>
+        <v>40.20243596528031</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>20.95841076203018</v>
+        <v>19.02230141015969</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>0.4169676386477593</v>
+        <v>0.5163316295136018</v>
       </c>
       <c r="K84" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L84" s="2" t="n">
         <v>0</v>
@@ -4924,31 +4924,31 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-0.2425739004286047</v>
+        <v>-0.2294428513595576</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>6914</v>
+        <v>7765</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>阜爾運通</t>
+          <t>中華資安</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>351.6461908947728</v>
+        <v>356.3177662010121</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>142.5</v>
+        <v>221.5</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
@@ -4959,16 +4959,16 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>46.91513569723856</v>
+        <v>38.25188507101979</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>9.301055141744916</v>
+        <v>20.95841076203018</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>0.6707749528069579</v>
+        <v>0.4169676386477593</v>
       </c>
       <c r="K85" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L85" s="2" t="n">
         <v>0</v>
@@ -4977,31 +4977,31 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>0.06783348748948009</v>
+        <v>-0.2425739004286047</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>7704</v>
+        <v>6873</v>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>明遠精密</t>
+          <t>泓德能源</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>345.9775013456459</v>
+        <v>355.1231478298612</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>60</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
@@ -5012,13 +5012,13 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>43.08052754930262</v>
+        <v>52.88983667921317</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>10.35003673546126</v>
+        <v>15.53961611986994</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>0.4674774304936214</v>
+        <v>0.569297001249601</v>
       </c>
       <c r="K86" s="2" t="n">
         <v>0</v>
@@ -5030,31 +5030,31 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-0.2137068832335129</v>
+        <v>1.068271818973007</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>7792</v>
+        <v>6914</v>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>安葆</t>
+          <t>阜爾運通</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>342.0459665854466</v>
+        <v>351.6461908947728</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>235.5</v>
+        <v>142.5</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
@@ -5065,16 +5065,16 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>33.84481336908068</v>
+        <v>46.91513569723856</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>21.04219704037088</v>
+        <v>9.301055141744916</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>0.4424815915393387</v>
+        <v>0.6707749528069579</v>
       </c>
       <c r="K87" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L87" s="2" t="n">
         <v>0</v>
@@ -5083,31 +5083,31 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>-1.195066356704928</v>
+        <v>0.06783348748948009</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>6855</v>
+        <v>7704</v>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>數泓科</t>
+          <t>明遠精密</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>337.4605930448236</v>
+        <v>345.9775013456459</v>
       </c>
       <c r="E88" s="2" t="n">
-        <v>122</v>
+        <v>60</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
@@ -5118,13 +5118,13 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>52.29651938628686</v>
+        <v>43.08052754930262</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>8.04114534922557</v>
+        <v>10.35003673546126</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>0.6924604135392959</v>
+        <v>0.4674774304936214</v>
       </c>
       <c r="K88" s="2" t="n">
         <v>0</v>
@@ -5136,31 +5136,31 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>0.4306449892046662</v>
+        <v>-0.2137068832335129</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>7728</v>
+        <v>6862</v>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>光焱科技</t>
+          <t>三集瑞-KY</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>332.3704498635813</v>
+        <v>345.0694609867115</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>654</v>
+        <v>181.5</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
@@ -5171,16 +5171,16 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>42.17218319386206</v>
+        <v>44.44859699964978</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>11.88058741850058</v>
+        <v>18.98089112724713</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>0.2558557370213209</v>
+        <v>0.3280607157287171</v>
       </c>
       <c r="K89" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L89" s="2" t="n">
         <v>0</v>
@@ -5189,31 +5189,31 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-2.451909478079361</v>
+        <v>-2.812789303812949</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>6923</v>
+        <v>7792</v>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>中台</t>
+          <t>安葆</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>331.4682919561231</v>
+        <v>342.0459665854466</v>
       </c>
       <c r="E90" s="2" t="n">
-        <v>75.40000000000001</v>
+        <v>235.5</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
@@ -5224,13 +5224,13 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>44.57626905084211</v>
+        <v>33.84481336908068</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>12.67822019372631</v>
+        <v>21.04219704037088</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>0.8082727665262706</v>
+        <v>0.4424815915393387</v>
       </c>
       <c r="K90" s="2" t="n">
         <v>0</v>
@@ -5242,31 +5242,31 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>0.2577025328151188</v>
+        <v>-1.195066356704928</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>6863</v>
+        <v>6855</v>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>永道-KY</t>
+          <t>數泓科</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>330.0321392910109</v>
+        <v>337.4605930448236</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>92.8</v>
+        <v>122</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
@@ -5277,16 +5277,16 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>41.40054904091114</v>
+        <v>52.29651938628686</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>20.6022182794955</v>
+        <v>8.04114534922557</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>0.1941587514346871</v>
+        <v>0.6924604135392959</v>
       </c>
       <c r="K91" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L91" s="2" t="n">
         <v>0</v>
@@ -5295,31 +5295,31 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>0.3684407432840513</v>
+        <v>0.4306449892046662</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>6937</v>
+        <v>7728</v>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>天虹</t>
+          <t>光焱科技</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>325.7484381391925</v>
+        <v>332.3704498635813</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>258.5</v>
+        <v>654</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
@@ -5330,16 +5330,16 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>41.58821044298968</v>
+        <v>42.17218319386206</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>11.66045158694848</v>
+        <v>11.88058741850058</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>0.5558910775457436</v>
+        <v>0.2558557370213209</v>
       </c>
       <c r="K92" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L92" s="2" t="n">
         <v>0</v>
@@ -5348,31 +5348,31 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-0.2642627748224893</v>
+        <v>-2.451909478079361</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>7751</v>
+        <v>6887</v>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>竑騰</t>
+          <t>寶綠特-KY</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>324.4173100399416</v>
+        <v>328.9710633676277</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>1295</v>
+        <v>33.8</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -5383,16 +5383,16 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>39.44757102375637</v>
+        <v>45.48886169883458</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>9.860766948779018</v>
+        <v>5.139339190518846</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>1.476844180607912</v>
+        <v>0.6399454679385927</v>
       </c>
       <c r="K93" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L93" s="2" t="n">
         <v>0</v>
@@ -5401,31 +5401,31 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>8.145777824020414</v>
+        <v>-0.1638936681527898</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>8047</v>
+        <v>7751</v>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>星雲</t>
+          <t>竑騰</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>322.5700999515211</v>
+        <v>324.4173100399416</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>44</v>
+        <v>1295</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
@@ -5436,16 +5436,16 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>39.94849770984634</v>
+        <v>39.44757102375637</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>7.110162534599978</v>
+        <v>9.860766948779018</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>0.8073288779987986</v>
+        <v>1.476844180607912</v>
       </c>
       <c r="K94" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L94" s="2" t="n">
         <v>0</v>
@@ -5454,31 +5454,31 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>-0.5620929104613687</v>
+        <v>8.145777824020414</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>8045</v>
+        <v>8047</v>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>達運光電</t>
+          <t>星雲</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>320.8412753222526</v>
+        <v>322.5700999515211</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>58.4</v>
+        <v>44</v>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
@@ -5489,13 +5489,13 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>38.28273749110956</v>
+        <v>39.94849770984634</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>11.24634823146596</v>
+        <v>7.110162534599978</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>0.7578615350408903</v>
+        <v>0.8073288779987986</v>
       </c>
       <c r="K95" s="2" t="n">
         <v>1</v>
@@ -5507,31 +5507,31 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>0.1666947706218837</v>
+        <v>-0.5620929104613687</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>6887</v>
+        <v>8045</v>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>寶綠特-KY</t>
+          <t>達運光電</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>308.9710633676277</v>
+        <v>320.8412753222526</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>33.8</v>
+        <v>58.4</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -5542,13 +5542,13 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>45.48886169883458</v>
+        <v>38.28273749110956</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>5.139339190518846</v>
+        <v>11.24634823146596</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>0.6399454679385927</v>
+        <v>0.7578615350408903</v>
       </c>
       <c r="K96" s="2" t="n">
         <v>1</v>
@@ -5560,31 +5560,31 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>-0.1638936681527898</v>
+        <v>0.1666947706218837</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>7736</v>
+        <v>6854</v>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>虎山</t>
+          <t>錼創科技-KY創</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>304.467327106767</v>
+        <v>307.9321804976679</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>70.40000000000001</v>
+        <v>113.5</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
@@ -5595,16 +5595,16 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>41.22229868003949</v>
+        <v>29.76518114133657</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>13.28760285875499</v>
+        <v>23.47971786607372</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>0.8334829319487406</v>
+        <v>1.527707214277649</v>
       </c>
       <c r="K97" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L97" s="2" t="n">
         <v>0</v>
@@ -5613,31 +5613,31 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>0.0114340746977891</v>
+        <v>-0.1925840124130724</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>8032</v>
+        <v>7736</v>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>光菱</t>
+          <t>虎山</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>301.7152547634907</v>
+        <v>304.467327106767</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>41.8</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5648,16 +5648,16 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>41.29813014855965</v>
+        <v>41.22229868003949</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>19.24859766789432</v>
+        <v>13.28760285875499</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>0.1251730459362888</v>
+        <v>0.8334829319487406</v>
       </c>
       <c r="K98" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L98" s="2" t="n">
         <v>0</v>
@@ -5666,31 +5666,31 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-0.4744961205503365</v>
+        <v>0.0114340746977891</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>6906</v>
+        <v>8032</v>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>現觀科</t>
+          <t>光菱</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
         <v/>
       </c>
       <c r="D99" s="2" t="n">
-        <v>298.577190325238</v>
+        <v>301.7152547634907</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>82</v>
+        <v>41.8</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
@@ -5701,16 +5701,16 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>39.51278555185927</v>
+        <v>41.29813014855965</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>17.85269472786651</v>
+        <v>19.24859766789432</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>0.3971803849544118</v>
+        <v>0.1251730459362888</v>
       </c>
       <c r="K99" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L99" s="2" t="n">
         <v>0</v>
@@ -5719,7 +5719,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-1.468828733260629</v>
+        <v>-0.4744961205503365</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5729,21 +5729,21 @@
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>6918</v>
+        <v>6906</v>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>愛派司</t>
+          <t>現觀科</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>297.0850751975527</v>
+        <v>298.577190325238</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>74.09999999999999</v>
+        <v>82</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
@@ -5754,13 +5754,13 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>52.23885075978043</v>
+        <v>39.51278555185927</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>13.4830962017074</v>
+        <v>17.85269472786651</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>0.4409605856337868</v>
+        <v>0.3971803849544118</v>
       </c>
       <c r="K100" s="2" t="n">
         <v>1</v>
@@ -5772,31 +5772,31 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>0.1896822961093553</v>
+        <v>-1.468828733260629</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
-        <v>6931</v>
+        <v>6918</v>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>青松健康</t>
+          <t>愛派司</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>296.6313441542502</v>
+        <v>297.0850751975527</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>39.75</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
@@ -5807,13 +5807,13 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>40.62086957529913</v>
+        <v>52.23885075978043</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>17.3503840018668</v>
+        <v>13.4830962017074</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>0.5679778257363548</v>
+        <v>0.4409605856337868</v>
       </c>
       <c r="K101" s="2" t="n">
         <v>1</v>
@@ -5825,7 +5825,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>0.068982221357753</v>
+        <v>0.1896822961093553</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5835,21 +5835,21 @@
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
-        <v>7721</v>
+        <v>6931</v>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>微程式</t>
+          <t>青松健康</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>294.8380842922334</v>
+        <v>296.6313441542502</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>71</v>
+        <v>39.75</v>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
@@ -5860,16 +5860,16 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>44.80168470812589</v>
+        <v>40.62086957529913</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>10.93154352012251</v>
+        <v>17.3503840018668</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>0.1445584497526122</v>
+        <v>0.5679778257363548</v>
       </c>
       <c r="K102" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L102" s="2" t="n">
         <v>0</v>
@@ -5878,31 +5878,31 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.2848709066211199</v>
+        <v>0.068982221357753</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
-        <v>6967</v>
+        <v>7721</v>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>汎瑋材料</t>
+          <t>微程式</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>294.6658513074201</v>
+        <v>294.8380842922334</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>69.40000000000001</v>
+        <v>71</v>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
@@ -5913,13 +5913,13 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>43.2632513968686</v>
+        <v>44.80168470812589</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>12.28915740397964</v>
+        <v>10.93154352012251</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>0.6501533329938837</v>
+        <v>0.1445584497526122</v>
       </c>
       <c r="K103" s="2" t="n">
         <v>0</v>
@@ -5931,31 +5931,31 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-0.1277832835988867</v>
+        <v>-0.2848709066211199</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
-        <v>6854</v>
+        <v>6967</v>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>錼創科技-KY創</t>
+          <t>汎瑋材料</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>287.9321804976679</v>
+        <v>294.6658513074201</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>113.5</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
@@ -5966,13 +5966,13 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>29.76518114133657</v>
+        <v>43.2632513968686</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>23.47971786607372</v>
+        <v>12.28915740397964</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>1.527707214277649</v>
+        <v>0.6501533329938837</v>
       </c>
       <c r="K104" s="2" t="n">
         <v>0</v>
@@ -5984,11 +5984,11 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-0.1925840124130724</v>
+        <v>-0.1277832835988867</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
@@ -6418,21 +6418,21 @@
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
-        <v>6908</v>
+        <v>6909</v>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>宏碁遊戲-創</t>
+          <t>創控</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>243.6464737414201</v>
+        <v>257.2207977387619</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>36.6</v>
+        <v>51.3</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
@@ -6443,13 +6443,13 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>35.67848240626194</v>
+        <v>44.84173236254644</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>16.1613569677956</v>
+        <v>16.43522249029083</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>0.9148933175702304</v>
+        <v>0.2418643455155242</v>
       </c>
       <c r="K113" s="2" t="n">
         <v>0</v>
@@ -6461,11 +6461,11 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-0.08735674367619881</v>
+        <v>-0.4028328879516456</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
@@ -6630,21 +6630,21 @@
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
-        <v>6921</v>
+        <v>6899</v>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>嘉雨思-創</t>
+          <t>創為精密</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
         <v/>
       </c>
       <c r="D117" s="2" t="n">
-        <v>226.6310574268157</v>
+        <v>218.6683684623978</v>
       </c>
       <c r="E117" s="2" t="n">
-        <v>68</v>
+        <v>54.7</v>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
@@ -6655,13 +6655,13 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>38.93343411596706</v>
+        <v>34.04625825395961</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>17.35227948019281</v>
+        <v>14.93820479383245</v>
       </c>
       <c r="J117" s="2" t="n">
-        <v>0.1668720314980874</v>
+        <v>0.9242118449439766</v>
       </c>
       <c r="K117" s="2" t="n">
         <v>0</v>
@@ -6673,31 +6673,31 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>0.2385507695230706</v>
+        <v>-0.3323764673576509</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
-        <v>6899</v>
+        <v>7749</v>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>創為精密</t>
+          <t>意騰-KY</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>218.6683684623978</v>
+        <v>216.15866189966</v>
       </c>
       <c r="E118" s="2" t="n">
-        <v>54.7</v>
+        <v>404</v>
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
@@ -6708,13 +6708,13 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>34.04625825395961</v>
+        <v>34.08472250739553</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>14.93820479383245</v>
+        <v>15.49490569347116</v>
       </c>
       <c r="J118" s="2" t="n">
-        <v>0.9242118449439766</v>
+        <v>0.2834734020563929</v>
       </c>
       <c r="K118" s="2" t="n">
         <v>0</v>
@@ -6726,31 +6726,31 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>-0.3323764673576509</v>
+        <v>-4.924311626850146</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
-        <v>6909</v>
+        <v>6885</v>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>創控</t>
+          <t>全福生技</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>217.220797738762</v>
+        <v>215.2736476833169</v>
       </c>
       <c r="E119" s="2" t="n">
-        <v>51.3</v>
+        <v>21.85</v>
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
@@ -6761,16 +6761,16 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>44.84173236254644</v>
+        <v>47.2964484181453</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>16.43522249029083</v>
+        <v>17.69471854733938</v>
       </c>
       <c r="J119" s="2" t="n">
-        <v>0.2418643455155242</v>
+        <v>0.4064297818704699</v>
       </c>
       <c r="K119" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L119" s="2" t="n">
         <v>0</v>
@@ -6779,31 +6779,31 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>-0.4028328879516456</v>
+        <v>0.06826108265377059</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
-        <v>7749</v>
+        <v>8044</v>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>意騰-KY</t>
+          <t>網家</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>216.15866189966</v>
+        <v>214.1764594044797</v>
       </c>
       <c r="E120" s="2" t="n">
-        <v>404</v>
+        <v>26.8</v>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
@@ -6814,13 +6814,13 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>34.08472250739553</v>
+        <v>41.52098254858291</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>15.49490569347116</v>
+        <v>14.18891225190132</v>
       </c>
       <c r="J120" s="2" t="n">
-        <v>0.2834734020563929</v>
+        <v>0.2486213192443414</v>
       </c>
       <c r="K120" s="2" t="n">
         <v>0</v>
@@ -6832,31 +6832,31 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-4.924311626850146</v>
+        <v>-0.3977575223101354</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
-        <v>6885</v>
+        <v>6908</v>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>全福生技</t>
+          <t>宏碁遊戲-創</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
         <v/>
       </c>
       <c r="D121" s="2" t="n">
-        <v>215.2736476833169</v>
+        <v>213.6464737414201</v>
       </c>
       <c r="E121" s="2" t="n">
-        <v>21.85</v>
+        <v>36.6</v>
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
@@ -6867,16 +6867,16 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>47.2964484181453</v>
+        <v>35.67848240626194</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>17.69471854733938</v>
+        <v>16.1613569677956</v>
       </c>
       <c r="J121" s="2" t="n">
-        <v>0.4064297818704699</v>
+        <v>0.9148933175702304</v>
       </c>
       <c r="K121" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L121" s="2" t="n">
         <v>0</v>
@@ -6885,7 +6885,7 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>0.06826108265377059</v>
+        <v>-0.08735674367619881</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
@@ -6895,21 +6895,21 @@
     </row>
     <row r="122">
       <c r="A122" s="2" t="n">
-        <v>8044</v>
+        <v>7730</v>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>網家</t>
+          <t>暉盛-創</t>
         </is>
       </c>
       <c r="C122" s="2" t="n">
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>214.1764594044797</v>
+        <v>209.1135777707526</v>
       </c>
       <c r="E122" s="2" t="n">
-        <v>26.8</v>
+        <v>183</v>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
@@ -6920,13 +6920,13 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>41.52098254858291</v>
+        <v>47.84907312567253</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>14.18891225190132</v>
+        <v>10.27348699793313</v>
       </c>
       <c r="J122" s="2" t="n">
-        <v>0.2486213192443414</v>
+        <v>0.9215102340619056</v>
       </c>
       <c r="K122" s="2" t="n">
         <v>0</v>
@@ -6938,31 +6938,31 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-0.3977575223101354</v>
+        <v>0.4485259988977426</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="n">
-        <v>7730</v>
+        <v>6953</v>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>暉盛-創</t>
+          <t>家碩</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
         <v/>
       </c>
       <c r="D123" s="2" t="n">
-        <v>209.1135777707526</v>
+        <v>202.7766110895432</v>
       </c>
       <c r="E123" s="2" t="n">
-        <v>183</v>
+        <v>228</v>
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
@@ -6973,13 +6973,13 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>47.84907312567253</v>
+        <v>43.79332010999956</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>10.27348699793313</v>
+        <v>12.77746564868914</v>
       </c>
       <c r="J123" s="2" t="n">
-        <v>0.9215102340619056</v>
+        <v>0.3861295447556247</v>
       </c>
       <c r="K123" s="2" t="n">
         <v>0</v>
@@ -6991,7 +6991,7 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>0.4485259988977426</v>
+        <v>0.2059930994131873</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
@@ -7001,21 +7001,21 @@
     </row>
     <row r="124">
       <c r="A124" s="2" t="n">
-        <v>6953</v>
+        <v>6859</v>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>家碩</t>
+          <t>伯特光</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
         <v/>
       </c>
       <c r="D124" s="2" t="n">
-        <v>202.7766110895432</v>
+        <v>202.4637793579379</v>
       </c>
       <c r="E124" s="2" t="n">
-        <v>228</v>
+        <v>120.5</v>
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
@@ -7026,13 +7026,13 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>43.79332010999956</v>
+        <v>42.96529548176591</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>12.77746564868914</v>
+        <v>15.9452175682549</v>
       </c>
       <c r="J124" s="2" t="n">
-        <v>0.3861295447556247</v>
+        <v>0.1066902570738212</v>
       </c>
       <c r="K124" s="2" t="n">
         <v>0</v>
@@ -7044,31 +7044,31 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>0.2059930994131873</v>
+        <v>-1.061681770343376</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, dealer_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="n">
-        <v>6859</v>
+        <v>6921</v>
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>伯特光</t>
+          <t>嘉雨思-創</t>
         </is>
       </c>
       <c r="C125" s="2" t="n">
         <v/>
       </c>
       <c r="D125" s="2" t="n">
-        <v>202.4637793579379</v>
+        <v>196.6310574268157</v>
       </c>
       <c r="E125" s="2" t="n">
-        <v>120.5</v>
+        <v>68</v>
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
@@ -7079,13 +7079,13 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>42.96529548176591</v>
+        <v>38.93343411596706</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>15.9452175682549</v>
+        <v>17.35227948019281</v>
       </c>
       <c r="J125" s="2" t="n">
-        <v>0.1066902570738212</v>
+        <v>0.1668720314980874</v>
       </c>
       <c r="K125" s="2" t="n">
         <v>0</v>
@@ -7097,11 +7097,11 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>-1.061681770343376</v>
+        <v>0.2385507695230706</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, dealer_buy_3d</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>

</xml_diff>